<commit_message>
remove password from acc
</commit_message>
<xml_diff>
--- a/accounts.xlsx
+++ b/accounts.xlsx
@@ -1,40 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
+  <si>
+    <t>Battletag</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Skill Rating</t>
+  </si>
+  <si>
+    <t>SR All Roles</t>
+  </si>
+  <si>
+    <t>KraftPunk#11658</t>
+  </si>
+  <si>
+    <t>NoSanaNoLife#1376</t>
+  </si>
+  <si>
+    <t>Daird#11322</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="0" formatCode="General"/>
+  </numFmts>
   <fonts count="3">
     <font>
+      <sz val="11"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
-      <color indexed="8"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color indexed="8"/>
       <name val="Helvetica Neue"/>
-      <color indexed="8"/>
-      <sz val="12"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
-      <color indexed="8"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -65,32 +91,32 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="0"/>
+  <tableStyles count="0"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="ff000000"/>
@@ -1163,86 +1189,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
+  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col width="8.851559999999999" customWidth="1" style="1" min="1" max="4"/>
-    <col width="8.851559999999999" customWidth="1" style="1" min="5" max="16384"/>
+    <col min="1" max="4" width="8.85156" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.85156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1" s="5">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Battletag</t>
-        </is>
+    <row r="1" ht="13.55" customHeight="1">
+      <c r="A1" t="s" s="2">
+        <v>0</v>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Password</t>
-        </is>
+      <c r="B1" t="s" s="2">
+        <v>1</v>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Skill Rating</t>
-        </is>
+      <c r="C1" t="s" s="2">
+        <v>2</v>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>SR All Roles</t>
-        </is>
+      <c r="D1" t="s" s="2">
+        <v>3</v>
       </c>
     </row>
-    <row r="2" ht="13.55" customHeight="1" s="5">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>KraftPunk#11658</t>
-        </is>
+    <row r="2" ht="13.55" customHeight="1">
+      <c r="A2" t="s" s="2">
+        <v>4</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>M000000w</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n">
+      <c r="B2" s="3"/>
+      <c r="C2" s="4">
         <v>4017</v>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="3"/>
     </row>
-    <row r="3" ht="13.55" customHeight="1" s="5">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>NoSanaNoLife#1376</t>
-        </is>
+    <row r="3" ht="13.55" customHeight="1">
+      <c r="A3" t="s" s="2">
+        <v>5</v>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
-    <row r="4" ht="13.55" customHeight="1" s="5">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Daird#11322</t>
-        </is>
+    <row r="4" ht="13.55" customHeight="1">
+      <c r="A4" t="s" s="2">
+        <v>6</v>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
opt for grabbing token out of environment
</commit_message>
<xml_diff>
--- a/accounts.xlsx
+++ b/accounts.xlsx
@@ -1,66 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
-  <si>
-    <t>Battletag</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>Skill Rating</t>
-  </si>
-  <si>
-    <t>SR All Roles</t>
-  </si>
-  <si>
-    <t>KraftPunk#11658</t>
-  </si>
-  <si>
-    <t>NoSanaNoLife#1376</t>
-  </si>
-  <si>
-    <t>Daird#11322</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
+      <name val="Calibri"/>
+      <color indexed="8"/>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color indexed="8"/>
       <sz val="14"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -91,32 +65,32 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="ff000000"/>
@@ -1189,59 +1163,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="4" width="8.85156" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col width="8.851559999999999" customWidth="1" style="1" min="1" max="4"/>
+    <col width="8.851559999999999" customWidth="1" style="1" min="5" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>0</v>
+    <row r="1" ht="13.55" customHeight="1" s="5">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Battletag</t>
+        </is>
       </c>
-      <c r="B1" t="s" s="2">
-        <v>1</v>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
       </c>
-      <c r="C1" t="s" s="2">
-        <v>2</v>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Skill Rating</t>
+        </is>
       </c>
-      <c r="D1" t="s" s="2">
-        <v>3</v>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>SR All Roles</t>
+        </is>
       </c>
     </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" t="s" s="2">
-        <v>4</v>
+    <row r="2" ht="13.55" customHeight="1" s="5">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KraftPunk#11658</t>
+        </is>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4">
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n">
         <v>4017</v>
       </c>
-      <c r="D2" s="3"/>
+      <c r="D2" s="4" t="n"/>
     </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" t="s" s="2">
-        <v>5</v>
+    <row r="3" ht="13.55" customHeight="1" s="5">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>NoSanaNoLife#1376</t>
+        </is>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" t="s" s="2">
-        <v>6</v>
+    <row r="4" ht="13.55" customHeight="1" s="5">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Daird#11322</t>
+        </is>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>